<commit_message>
rail panels: add xtm short handstop with index panel stats
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changes/rail-panels.xlsx
+++ b/changes/rail-panels.xlsx
@@ -921,7 +921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O39"/>
+  <dimension ref="A1:O40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="27.140625" customWidth="1" min="2" max="2"/>
@@ -1373,42 +1373,41 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n"/>
-      <c r="B14" s="1" t="n"/>
-      <c r="C14" s="1" t="n"/>
-      <c r="D14" s="1" t="n"/>
-      <c r="E14" s="1" t="n"/>
-      <c r="F14" s="1" t="n"/>
-      <c r="G14" s="1" t="n"/>
-      <c r="H14" s="1" t="n"/>
-      <c r="I14" s="1" t="n"/>
-      <c r="J14" s="1" t="n"/>
-      <c r="K14" s="1" t="n"/>
-      <c r="L14" s="1" t="n"/>
-      <c r="M14" s="1" t="n"/>
-      <c r="N14" s="1" t="n"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>magtap_xtm_enhanced_short_handstop_1</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Magtap XTM Enhanced Short Handstop Piece</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-2</v>
+      </c>
+      <c r="M14" t="n">
+        <v>50</v>
+      </c>
       <c r="O14">
         <f>C14-D14*20-E14*0.8-F14*0.6-H14*10+I14*15+J14/200-M14*5</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>axtell_defense_3inch_picatinny_rail_panel</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
-        <is>
-          <t>Axtell Defense 3 inch Picatinny</t>
-        </is>
-      </c>
-      <c r="C15" s="1" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="D15" s="1" t="n">
-        <v>0.04</v>
-      </c>
+      <c r="A15" s="1" t="n"/>
+      <c r="B15" s="1" t="n"/>
+      <c r="C15" s="1" t="n"/>
+      <c r="D15" s="1" t="n"/>
       <c r="E15" s="1" t="n"/>
       <c r="F15" s="1" t="n"/>
       <c r="G15" s="1" t="n"/>
@@ -1417,9 +1416,7 @@
       <c r="J15" s="1" t="n"/>
       <c r="K15" s="1" t="n"/>
       <c r="L15" s="1" t="n"/>
-      <c r="M15" s="1" t="n">
-        <v>300</v>
-      </c>
+      <c r="M15" s="1" t="n"/>
       <c r="N15" s="1" t="n"/>
       <c r="O15">
         <f>C15-D15*20-E15*0.8-F15*0.6-H15*10+I15*15+J15/200-M15*5</f>
@@ -1429,19 +1426,19 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>axtell_defense_5inch_picatinny_rail_panel</t>
+          <t>axtell_defense_3inch_picatinny_rail_panel</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>Axtell Defense 5 inch Picatinny</t>
+          <t>Axtell Defense 3 inch Picatinny</t>
         </is>
       </c>
       <c r="C16" s="1" t="n">
-        <v>2</v>
+        <v>1.33</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E16" s="1" t="n"/>
       <c r="F16" s="1" t="n"/>
@@ -1452,7 +1449,7 @@
       <c r="K16" s="1" t="n"/>
       <c r="L16" s="1" t="n"/>
       <c r="M16" s="1" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="N16" s="1" t="n"/>
       <c r="O16">
@@ -1463,19 +1460,19 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>axtell_defense_7inch_picatinny_rail_panel</t>
+          <t>axtell_defense_5inch_picatinny_rail_panel</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>Axtell Defense 7 inch Picatinny</t>
+          <t>Axtell Defense 5 inch Picatinny</t>
         </is>
       </c>
       <c r="C17" s="1" t="n">
-        <v>2.66</v>
+        <v>2</v>
       </c>
       <c r="D17" s="1" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="E17" s="1" t="n"/>
       <c r="F17" s="1" t="n"/>
@@ -1486,7 +1483,7 @@
       <c r="K17" s="1" t="n"/>
       <c r="L17" s="1" t="n"/>
       <c r="M17" s="1" t="n">
-        <v>700</v>
+        <v>500</v>
       </c>
       <c r="N17" s="1" t="n"/>
       <c r="O17">
@@ -1495,10 +1492,22 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n"/>
-      <c r="B18" s="1" t="n"/>
-      <c r="C18" s="1" t="n"/>
-      <c r="D18" s="1" t="n"/>
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>axtell_defense_7inch_picatinny_rail_panel</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>Axtell Defense 7 inch Picatinny</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="D18" s="1" t="n">
+        <v>0.08</v>
+      </c>
       <c r="E18" s="1" t="n"/>
       <c r="F18" s="1" t="n"/>
       <c r="G18" s="1" t="n"/>
@@ -1507,7 +1516,9 @@
       <c r="J18" s="1" t="n"/>
       <c r="K18" s="1" t="n"/>
       <c r="L18" s="1" t="n"/>
-      <c r="M18" s="1" t="n"/>
+      <c r="M18" s="1" t="n">
+        <v>700</v>
+      </c>
       <c r="N18" s="1" t="n"/>
       <c r="O18">
         <f>C18-D18*20-E18*0.8-F18*0.6-H18*10+I18*15+J18/200-M18*5</f>
@@ -1515,22 +1526,10 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>veles_npn_2_half_rail_cover</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
-        <is>
-          <t>Veles NPN-2 Half</t>
-        </is>
-      </c>
-      <c r="C19" s="1" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="D19" s="1" t="n">
-        <v>0.02</v>
-      </c>
+      <c r="A19" s="1" t="n"/>
+      <c r="B19" s="1" t="n"/>
+      <c r="C19" s="1" t="n"/>
+      <c r="D19" s="1" t="n"/>
       <c r="E19" s="1" t="n"/>
       <c r="F19" s="1" t="n"/>
       <c r="G19" s="1" t="n"/>
@@ -1539,9 +1538,7 @@
       <c r="J19" s="1" t="n"/>
       <c r="K19" s="1" t="n"/>
       <c r="L19" s="1" t="n"/>
-      <c r="M19" s="1" t="n">
-        <v>300</v>
-      </c>
+      <c r="M19" s="1" t="n"/>
       <c r="N19" s="1" t="n"/>
       <c r="O19">
         <f>C19-D19*20-E19*0.8-F19*0.6-H19*10+I19*15+J19/200-M19*5</f>
@@ -1551,19 +1548,19 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>veles_npn_2_rail_cover</t>
+          <t>veles_npn_2_half_rail_cover</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>Veles NPN-2</t>
+          <t>Veles NPN-2 Half</t>
         </is>
       </c>
       <c r="C20" s="1" t="n">
-        <v>1</v>
+        <v>0.66</v>
       </c>
       <c r="D20" s="1" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="E20" s="1" t="n"/>
       <c r="F20" s="1" t="n"/>
@@ -1574,7 +1571,7 @@
       <c r="K20" s="1" t="n"/>
       <c r="L20" s="1" t="n"/>
       <c r="M20" s="1" t="n">
-        <v>750</v>
+        <v>300</v>
       </c>
       <c r="N20" s="1" t="n"/>
       <c r="O20">
@@ -1583,10 +1580,22 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n"/>
-      <c r="B21" s="1" t="n"/>
-      <c r="C21" s="1" t="n"/>
-      <c r="D21" s="1" t="n"/>
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>veles_npn_2_rail_cover</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t>Veles NPN-2</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="1" t="n">
+        <v>0.03</v>
+      </c>
       <c r="E21" s="1" t="n"/>
       <c r="F21" s="1" t="n"/>
       <c r="G21" s="1" t="n"/>
@@ -1595,7 +1604,9 @@
       <c r="J21" s="1" t="n"/>
       <c r="K21" s="1" t="n"/>
       <c r="L21" s="1" t="n"/>
-      <c r="M21" s="1" t="n"/>
+      <c r="M21" s="1" t="n">
+        <v>750</v>
+      </c>
       <c r="N21" s="1" t="n"/>
       <c r="O21">
         <f>C21-D21*20-E21*0.8-F21*0.6-H21*10+I21*15+J21/200-M21*5</f>
@@ -1603,22 +1614,10 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>equinox_ex_mlok_cover</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
-        <is>
-          <t>Arrow AX</t>
-        </is>
-      </c>
-      <c r="C22" s="1" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="D22" s="1" t="n">
-        <v>0.02</v>
-      </c>
+      <c r="A22" s="1" t="n"/>
+      <c r="B22" s="1" t="n"/>
+      <c r="C22" s="1" t="n"/>
+      <c r="D22" s="1" t="n"/>
       <c r="E22" s="1" t="n"/>
       <c r="F22" s="1" t="n"/>
       <c r="G22" s="1" t="n"/>
@@ -1627,9 +1626,7 @@
       <c r="J22" s="1" t="n"/>
       <c r="K22" s="1" t="n"/>
       <c r="L22" s="1" t="n"/>
-      <c r="M22" s="1" t="n">
-        <v>100</v>
-      </c>
+      <c r="M22" s="1" t="n"/>
       <c r="N22" s="1" t="n"/>
       <c r="O22">
         <f>C22-D22*20-E22*0.8-F22*0.6-H22*10+I22*15+J22/200-M22*5</f>
@@ -1639,12 +1636,12 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>equinox_ex_mlok_cover_flipped</t>
+          <t>equinox_ex_mlok_cover</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t>Arrow AX Flipped</t>
+          <t>Arrow AX</t>
         </is>
       </c>
       <c r="C23" s="1" t="n">
@@ -1671,10 +1668,22 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n"/>
-      <c r="B24" s="1" t="n"/>
-      <c r="C24" s="1" t="n"/>
-      <c r="D24" s="1" t="n"/>
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>equinox_ex_mlok_cover_flipped</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>Arrow AX Flipped</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="D24" s="1" t="n">
+        <v>0.02</v>
+      </c>
       <c r="E24" s="1" t="n"/>
       <c r="F24" s="1" t="n"/>
       <c r="G24" s="1" t="n"/>
@@ -1683,7 +1692,9 @@
       <c r="J24" s="1" t="n"/>
       <c r="K24" s="1" t="n"/>
       <c r="L24" s="1" t="n"/>
-      <c r="M24" s="1" t="n"/>
+      <c r="M24" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="N24" s="1" t="n"/>
       <c r="O24">
         <f>C24-D24*20-E24*0.8-F24*0.6-H24*10+I24*15+J24/200-M24*5</f>
@@ -1691,22 +1702,10 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>magtap_type_1_1slot_mlok_cover</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
-        <is>
-          <t>Magtap Type1 1 Slot MLOK</t>
-        </is>
-      </c>
-      <c r="C25" s="1" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="D25" s="1" t="n">
-        <v>0.02</v>
-      </c>
+      <c r="A25" s="1" t="n"/>
+      <c r="B25" s="1" t="n"/>
+      <c r="C25" s="1" t="n"/>
+      <c r="D25" s="1" t="n"/>
       <c r="E25" s="1" t="n"/>
       <c r="F25" s="1" t="n"/>
       <c r="G25" s="1" t="n"/>
@@ -1715,9 +1714,7 @@
       <c r="J25" s="1" t="n"/>
       <c r="K25" s="1" t="n"/>
       <c r="L25" s="1" t="n"/>
-      <c r="M25" s="1" t="n">
-        <v>100</v>
-      </c>
+      <c r="M25" s="1" t="n"/>
       <c r="N25" s="1" t="n"/>
       <c r="O25">
         <f>C25-D25*20-E25*0.8-F25*0.6-H25*10+I25*15+J25/200-M25*5</f>
@@ -1727,19 +1724,19 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>magtap_type_1_3_slot_mlok_cover</t>
+          <t>magtap_type_1_1slot_mlok_cover</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t>Magtap Type1 3 Slot MLOK</t>
+          <t>Magtap Type1 1 Slot MLOK</t>
         </is>
       </c>
       <c r="C26" s="1" t="n">
-        <v>1.66</v>
+        <v>0.66</v>
       </c>
       <c r="D26" s="1" t="n">
-        <v>0.05</v>
+        <v>0.02</v>
       </c>
       <c r="E26" s="1" t="n"/>
       <c r="F26" s="1" t="n"/>
@@ -1750,7 +1747,7 @@
       <c r="K26" s="1" t="n"/>
       <c r="L26" s="1" t="n"/>
       <c r="M26" s="1" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="N26" s="1" t="n"/>
       <c r="O26">
@@ -1761,19 +1758,19 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>magtap_type_1_6slot_mlok_cover</t>
+          <t>magtap_type_1_3_slot_mlok_cover</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>Magtap Type1 6 Slot MLOK</t>
+          <t>Magtap Type1 3 Slot MLOK</t>
         </is>
       </c>
       <c r="C27" s="1" t="n">
-        <v>3</v>
+        <v>1.66</v>
       </c>
       <c r="D27" s="1" t="n">
-        <v>0.09</v>
+        <v>0.05</v>
       </c>
       <c r="E27" s="1" t="n"/>
       <c r="F27" s="1" t="n"/>
@@ -1784,7 +1781,7 @@
       <c r="K27" s="1" t="n"/>
       <c r="L27" s="1" t="n"/>
       <c r="M27" s="1" t="n">
-        <v>900</v>
+        <v>300</v>
       </c>
       <c r="N27" s="1" t="n"/>
       <c r="O27">
@@ -1793,10 +1790,22 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n"/>
-      <c r="B28" s="1" t="n"/>
-      <c r="C28" s="1" t="n"/>
-      <c r="D28" s="1" t="n"/>
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>magtap_type_1_6slot_mlok_cover</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t>Magtap Type1 6 Slot MLOK</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>0.09</v>
+      </c>
       <c r="E28" s="1" t="n"/>
       <c r="F28" s="1" t="n"/>
       <c r="G28" s="1" t="n"/>
@@ -1805,7 +1814,9 @@
       <c r="J28" s="1" t="n"/>
       <c r="K28" s="1" t="n"/>
       <c r="L28" s="1" t="n"/>
-      <c r="M28" s="1" t="n"/>
+      <c r="M28" s="1" t="n">
+        <v>900</v>
+      </c>
       <c r="N28" s="1" t="n"/>
       <c r="O28">
         <f>C28-D28*20-E28*0.8-F28*0.6-H28*10+I28*15+J28/200-M28*5</f>
@@ -1813,22 +1824,10 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>magtap_type_2_half_mlok_cover</t>
-        </is>
-      </c>
-      <c r="B29" s="1" t="inlineStr">
-        <is>
-          <t>Magtap Type2 Half Cover</t>
-        </is>
-      </c>
-      <c r="C29" s="1" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="D29" s="1" t="n">
-        <v>0.01</v>
-      </c>
+      <c r="A29" s="1" t="n"/>
+      <c r="B29" s="1" t="n"/>
+      <c r="C29" s="1" t="n"/>
+      <c r="D29" s="1" t="n"/>
       <c r="E29" s="1" t="n"/>
       <c r="F29" s="1" t="n"/>
       <c r="G29" s="1" t="n"/>
@@ -1837,9 +1836,7 @@
       <c r="J29" s="1" t="n"/>
       <c r="K29" s="1" t="n"/>
       <c r="L29" s="1" t="n"/>
-      <c r="M29" s="1" t="n">
-        <v>100</v>
-      </c>
+      <c r="M29" s="1" t="n"/>
       <c r="N29" s="1" t="n"/>
       <c r="O29">
         <f>C29-D29*20-E29*0.8-F29*0.6-H29*10+I29*15+J29/200-M29*5</f>
@@ -1849,19 +1846,19 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>magtap_type_2_mlok_cover</t>
+          <t>magtap_type_2_half_mlok_cover</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
-          <t>Magtap Type2 Cover</t>
+          <t>Magtap Type2 Half Cover</t>
         </is>
       </c>
       <c r="C30" s="1" t="n">
-        <v>0.66</v>
+        <v>0.33</v>
       </c>
       <c r="D30" s="1" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="E30" s="1" t="n"/>
       <c r="F30" s="1" t="n"/>
@@ -1872,7 +1869,7 @@
       <c r="K30" s="1" t="n"/>
       <c r="L30" s="1" t="n"/>
       <c r="M30" s="1" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="N30" s="1" t="n"/>
       <c r="O30">
@@ -1881,10 +1878,22 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n"/>
-      <c r="B31" s="1" t="n"/>
-      <c r="C31" s="1" t="n"/>
-      <c r="D31" s="1" t="n"/>
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>magtap_type_2_mlok_cover</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
+        <is>
+          <t>Magtap Type2 Cover</t>
+        </is>
+      </c>
+      <c r="C31" s="1" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="D31" s="1" t="n">
+        <v>0.02</v>
+      </c>
       <c r="E31" s="1" t="n"/>
       <c r="F31" s="1" t="n"/>
       <c r="G31" s="1" t="n"/>
@@ -1893,7 +1902,9 @@
       <c r="J31" s="1" t="n"/>
       <c r="K31" s="1" t="n"/>
       <c r="L31" s="1" t="n"/>
-      <c r="M31" s="1" t="n"/>
+      <c r="M31" s="1" t="n">
+        <v>200</v>
+      </c>
       <c r="N31" s="1" t="n"/>
       <c r="O31">
         <f>C31-D31*20-E31*0.8-F31*0.6-H31*10+I31*15+J31/200-M31*5</f>
@@ -1901,22 +1912,10 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="inlineStr">
-        <is>
-          <t>ecm_ecmr_1_slot_mlok_rail_panel</t>
-        </is>
-      </c>
-      <c r="B32" s="1" t="inlineStr">
-        <is>
-          <t>ECM ECMR 1 Slot</t>
-        </is>
-      </c>
-      <c r="C32" s="1" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="D32" s="1" t="n">
-        <v>0.01</v>
-      </c>
+      <c r="A32" s="1" t="n"/>
+      <c r="B32" s="1" t="n"/>
+      <c r="C32" s="1" t="n"/>
+      <c r="D32" s="1" t="n"/>
       <c r="E32" s="1" t="n"/>
       <c r="F32" s="1" t="n"/>
       <c r="G32" s="1" t="n"/>
@@ -1925,9 +1924,7 @@
       <c r="J32" s="1" t="n"/>
       <c r="K32" s="1" t="n"/>
       <c r="L32" s="1" t="n"/>
-      <c r="M32" s="1" t="n">
-        <v>200</v>
-      </c>
+      <c r="M32" s="1" t="n"/>
       <c r="N32" s="1" t="n"/>
       <c r="O32">
         <f>C32-D32*20-E32*0.8-F32*0.6-H32*10+I32*15+J32/200-M32*5</f>
@@ -1937,19 +1934,19 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>ecm_ecmr_3_slot_mlok_rail_panel</t>
+          <t>ecm_ecmr_1_slot_mlok_rail_panel</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t>ECM ECMR 3 Slot</t>
+          <t>ECM ECMR 1 Slot</t>
         </is>
       </c>
       <c r="C33" s="1" t="n">
-        <v>1</v>
+        <v>0.33</v>
       </c>
       <c r="D33" s="1" t="n">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="E33" s="1" t="n"/>
       <c r="F33" s="1" t="n"/>
@@ -1960,7 +1957,7 @@
       <c r="K33" s="1" t="n"/>
       <c r="L33" s="1" t="n"/>
       <c r="M33" s="1" t="n">
-        <v>600</v>
+        <v>200</v>
       </c>
       <c r="N33" s="1" t="n"/>
       <c r="O33">
@@ -1971,19 +1968,19 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>ecm_ecmr_7_slot_mlok_rail_panel</t>
+          <t>ecm_ecmr_3_slot_mlok_rail_panel</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t>ECM ECMR 7 Slot</t>
+          <t>ECM ECMR 3 Slot</t>
         </is>
       </c>
       <c r="C34" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D34" s="1" t="n">
-        <v>0.06</v>
+        <v>0.03</v>
       </c>
       <c r="E34" s="1" t="n"/>
       <c r="F34" s="1" t="n"/>
@@ -1994,7 +1991,7 @@
       <c r="K34" s="1" t="n"/>
       <c r="L34" s="1" t="n"/>
       <c r="M34" s="1" t="n">
-        <v>1000</v>
+        <v>600</v>
       </c>
       <c r="N34" s="1" t="n"/>
       <c r="O34">
@@ -2003,10 +2000,22 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n"/>
-      <c r="B35" s="1" t="n"/>
-      <c r="C35" s="1" t="n"/>
-      <c r="D35" s="1" t="n"/>
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>ecm_ecmr_7_slot_mlok_rail_panel</t>
+        </is>
+      </c>
+      <c r="B35" s="1" t="inlineStr">
+        <is>
+          <t>ECM ECMR 7 Slot</t>
+        </is>
+      </c>
+      <c r="C35" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D35" s="1" t="n">
+        <v>0.06</v>
+      </c>
       <c r="E35" s="1" t="n"/>
       <c r="F35" s="1" t="n"/>
       <c r="G35" s="1" t="n"/>
@@ -2015,8 +2024,14 @@
       <c r="J35" s="1" t="n"/>
       <c r="K35" s="1" t="n"/>
       <c r="L35" s="1" t="n"/>
-      <c r="M35" s="1" t="n"/>
+      <c r="M35" s="1" t="n">
+        <v>1000</v>
+      </c>
       <c r="N35" s="1" t="n"/>
+      <c r="O35">
+        <f>C35-D35*20-E35*0.8-F35*0.6-H35*10+I35*15+J35/200-M35*5</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n"/>
@@ -2033,6 +2048,10 @@
       <c r="L36" s="1" t="n"/>
       <c r="M36" s="1" t="n"/>
       <c r="N36" s="1" t="n"/>
+      <c r="O36">
+        <f>C36-D36*20-E36*0.8-F36*0.6-H36*10+I36*15+J36/200-M36*5</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n"/>
@@ -2049,6 +2068,10 @@
       <c r="L37" s="1" t="n"/>
       <c r="M37" s="1" t="n"/>
       <c r="N37" s="1" t="n"/>
+      <c r="O37">
+        <f>C37-D37*20-E37*0.8-F37*0.6-H37*10+I37*15+J37/200-M37*5</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n"/>
@@ -2065,6 +2088,10 @@
       <c r="L38" s="1" t="n"/>
       <c r="M38" s="1" t="n"/>
       <c r="N38" s="1" t="n"/>
+      <c r="O38">
+        <f>C38-D38*20-E38*0.8-F38*0.6-H38*10+I38*15+J38/200-M38*5</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n"/>
@@ -2081,6 +2108,30 @@
       <c r="L39" s="1" t="n"/>
       <c r="M39" s="1" t="n"/>
       <c r="N39" s="1" t="n"/>
+      <c r="O39">
+        <f>C39-D39*20-E39*0.8-F39*0.6-H39*10+I39*15+J39/200-M39*5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n"/>
+      <c r="B40" s="1" t="n"/>
+      <c r="C40" s="1" t="n"/>
+      <c r="D40" s="1" t="n"/>
+      <c r="E40" s="1" t="n"/>
+      <c r="F40" s="1" t="n"/>
+      <c r="G40" s="1" t="n"/>
+      <c r="H40" s="1" t="n"/>
+      <c r="I40" s="1" t="n"/>
+      <c r="J40" s="1" t="n"/>
+      <c r="K40" s="1" t="n"/>
+      <c r="L40" s="1" t="n"/>
+      <c r="M40" s="1" t="n"/>
+      <c r="N40" s="1" t="n"/>
+      <c r="O40">
+        <f>C40-D40*20-E40*0.8-F40*0.6-H40*10+I40*15+J40/200-M40*5</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
rail panel sheet: fix strength formula, add CGR panels
</commit_message>
<xml_diff>
--- a/changes/rail-panels.xlsx
+++ b/changes/rail-panels.xlsx
@@ -921,7 +921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O39"/>
+  <dimension ref="A1:O49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="27.140625" customWidth="1" min="2" max="2"/>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="N3" s="1" t="n"/>
       <c r="O3">
-        <f>C3-D3*20-E3*0.8-F3*0.6-H3*10+I3*15+J3/200-M3*5</f>
+        <f>C3-D3*20-E3*0.8-F3*0.6-H3*10+I3*15+J3/200-N3*5</f>
         <v/>
       </c>
     </row>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="N4" s="1" t="n"/>
       <c r="O4">
-        <f>C4-D4*20-E4*0.8-F4*0.6-H4*10+I4*15+J4/200-M4*5</f>
+        <f>C4-D4*20-E4*0.8-F4*0.6-H4*10+I4*15+J4/200-N4*5</f>
         <v/>
       </c>
     </row>
@@ -1110,7 +1110,7 @@
       </c>
       <c r="N5" s="1" t="n"/>
       <c r="O5">
-        <f>C5-D5*20-E5*0.8-F5*0.6-H5*10+I5*15+J5/200-M5*5</f>
+        <f>C5-D5*20-E5*0.8-F5*0.6-H5*10+I5*15+J5/200-N5*5</f>
         <v/>
       </c>
     </row>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="N6" s="1" t="n"/>
       <c r="O6">
-        <f>C6-D6*20-E6*0.8-F6*0.6-H6*10+I6*15+J6/200-M6*5</f>
+        <f>C6-D6*20-E6*0.8-F6*0.6-H6*10+I6*15+J6/200-N6*5</f>
         <v/>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="N7" s="1" t="n"/>
       <c r="O7">
-        <f>C7-D7*20-E7*0.8-F7*0.6-H7*10+I7*15+J7/200-M7*5</f>
+        <f>C7-D7*20-E7*0.8-F7*0.6-H7*10+I7*15+J7/200-N7*5</f>
         <v/>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="N8" s="1" t="n"/>
       <c r="O8">
-        <f>C8-D8*20-E8*0.8-F8*0.6-H8*10+I8*15+J8/200-M8*5</f>
+        <f>C8-D8*20-E8*0.8-F8*0.6-H8*10+I8*15+J8/200-N8*5</f>
         <v/>
       </c>
     </row>
@@ -1232,7 +1232,7 @@
       <c r="M9" s="1" t="n"/>
       <c r="N9" s="1" t="n"/>
       <c r="O9">
-        <f>C9-D9*20-E9*0.8-F9*0.6-H9*10+I9*15+J9/200-M9*5</f>
+        <f>C9-D9*20-E9*0.8-F9*0.6-H9*10+I9*15+J9/200-N9*5</f>
         <v/>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="N10" s="1" t="n"/>
       <c r="O10">
-        <f>C10-D10*20-E10*0.8-F10*0.6-H10*10+I10*15+J10/200-M10*5</f>
+        <f>C10-D10*20-E10*0.8-F10*0.6-H10*10+I10*15+J10/200-N10*5</f>
         <v/>
       </c>
     </row>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="N11" s="1" t="n"/>
       <c r="O11">
-        <f>C11-D11*20-E11*0.8-F11*0.6-H11*10+I11*15+J11/200-M11*5</f>
+        <f>C11-D11*20-E11*0.8-F11*0.6-H11*10+I11*15+J11/200-N11*5</f>
         <v/>
       </c>
     </row>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="N12" s="1" t="n"/>
       <c r="O12">
-        <f>C12-D12*20-E12*0.8-F12*0.6-H12*10+I12*15+J12/200-M12*5</f>
+        <f>C12-D12*20-E12*0.8-F12*0.6-H12*10+I12*15+J12/200-N12*5</f>
         <v/>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="N13" s="1" t="n"/>
       <c r="O13">
-        <f>C13-D13*20-E13*0.8-F13*0.6-H13*10+I13*15+J13/200-M13*5</f>
+        <f>C13-D13*20-E13*0.8-F13*0.6-H13*10+I13*15+J13/200-N13*5</f>
         <v/>
       </c>
     </row>
@@ -1388,7 +1388,7 @@
       <c r="M14" s="1" t="n"/>
       <c r="N14" s="1" t="n"/>
       <c r="O14">
-        <f>C14-D14*20-E14*0.8-F14*0.6-H14*10+I14*15+J14/200-M14*5</f>
+        <f>C14-D14*20-E14*0.8-F14*0.6-H14*10+I14*15+J14/200-N14*5</f>
         <v/>
       </c>
     </row>
@@ -1422,7 +1422,7 @@
       </c>
       <c r="N15" s="1" t="n"/>
       <c r="O15">
-        <f>C15-D15*20-E15*0.8-F15*0.6-H15*10+I15*15+J15/200-M15*5</f>
+        <f>C15-D15*20-E15*0.8-F15*0.6-H15*10+I15*15+J15/200-N15*5</f>
         <v/>
       </c>
     </row>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="N16" s="1" t="n"/>
       <c r="O16">
-        <f>C16-D16*20-E16*0.8-F16*0.6-H16*10+I16*15+J16/200-M16*5</f>
+        <f>C16-D16*20-E16*0.8-F16*0.6-H16*10+I16*15+J16/200-N16*5</f>
         <v/>
       </c>
     </row>
@@ -1490,7 +1490,7 @@
       </c>
       <c r="N17" s="1" t="n"/>
       <c r="O17">
-        <f>C17-D17*20-E17*0.8-F17*0.6-H17*10+I17*15+J17/200-M17*5</f>
+        <f>C17-D17*20-E17*0.8-F17*0.6-H17*10+I17*15+J17/200-N17*5</f>
         <v/>
       </c>
     </row>
@@ -1510,7 +1510,7 @@
       <c r="M18" s="1" t="n"/>
       <c r="N18" s="1" t="n"/>
       <c r="O18">
-        <f>C18-D18*20-E18*0.8-F18*0.6-H18*10+I18*15+J18/200-M18*5</f>
+        <f>C18-D18*20-E18*0.8-F18*0.6-H18*10+I18*15+J18/200-N18*5</f>
         <v/>
       </c>
     </row>
@@ -1544,7 +1544,7 @@
       </c>
       <c r="N19" s="1" t="n"/>
       <c r="O19">
-        <f>C19-D19*20-E19*0.8-F19*0.6-H19*10+I19*15+J19/200-M19*5</f>
+        <f>C19-D19*20-E19*0.8-F19*0.6-H19*10+I19*15+J19/200-N19*5</f>
         <v/>
       </c>
     </row>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="N20" s="1" t="n"/>
       <c r="O20">
-        <f>C20-D20*20-E20*0.8-F20*0.6-H20*10+I20*15+J20/200-M20*5</f>
+        <f>C20-D20*20-E20*0.8-F20*0.6-H20*10+I20*15+J20/200-N20*5</f>
         <v/>
       </c>
     </row>
@@ -1598,7 +1598,7 @@
       <c r="M21" s="1" t="n"/>
       <c r="N21" s="1" t="n"/>
       <c r="O21">
-        <f>C21-D21*20-E21*0.8-F21*0.6-H21*10+I21*15+J21/200-M21*5</f>
+        <f>C21-D21*20-E21*0.8-F21*0.6-H21*10+I21*15+J21/200-N21*5</f>
         <v/>
       </c>
     </row>
@@ -1632,7 +1632,7 @@
       </c>
       <c r="N22" s="1" t="n"/>
       <c r="O22">
-        <f>C22-D22*20-E22*0.8-F22*0.6-H22*10+I22*15+J22/200-M22*5</f>
+        <f>C22-D22*20-E22*0.8-F22*0.6-H22*10+I22*15+J22/200-N22*5</f>
         <v/>
       </c>
     </row>
@@ -1666,7 +1666,7 @@
       </c>
       <c r="N23" s="1" t="n"/>
       <c r="O23">
-        <f>C23-D23*20-E23*0.8-F23*0.6-H23*10+I23*15+J23/200-M23*5</f>
+        <f>C23-D23*20-E23*0.8-F23*0.6-H23*10+I23*15+J23/200-N23*5</f>
         <v/>
       </c>
     </row>
@@ -1686,7 +1686,7 @@
       <c r="M24" s="1" t="n"/>
       <c r="N24" s="1" t="n"/>
       <c r="O24">
-        <f>C24-D24*20-E24*0.8-F24*0.6-H24*10+I24*15+J24/200-M24*5</f>
+        <f>C24-D24*20-E24*0.8-F24*0.6-H24*10+I24*15+J24/200-N24*5</f>
         <v/>
       </c>
     </row>
@@ -1720,7 +1720,7 @@
       </c>
       <c r="N25" s="1" t="n"/>
       <c r="O25">
-        <f>C25-D25*20-E25*0.8-F25*0.6-H25*10+I25*15+J25/200-M25*5</f>
+        <f>C25-D25*20-E25*0.8-F25*0.6-H25*10+I25*15+J25/200-N25*5</f>
         <v/>
       </c>
     </row>
@@ -1754,7 +1754,7 @@
       </c>
       <c r="N26" s="1" t="n"/>
       <c r="O26">
-        <f>C26-D26*20-E26*0.8-F26*0.6-H26*10+I26*15+J26/200-M26*5</f>
+        <f>C26-D26*20-E26*0.8-F26*0.6-H26*10+I26*15+J26/200-N26*5</f>
         <v/>
       </c>
     </row>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="N27" s="1" t="n"/>
       <c r="O27">
-        <f>C27-D27*20-E27*0.8-F27*0.6-H27*10+I27*15+J27/200-M27*5</f>
+        <f>C27-D27*20-E27*0.8-F27*0.6-H27*10+I27*15+J27/200-N27*5</f>
         <v/>
       </c>
     </row>
@@ -1808,7 +1808,7 @@
       <c r="M28" s="1" t="n"/>
       <c r="N28" s="1" t="n"/>
       <c r="O28">
-        <f>C28-D28*20-E28*0.8-F28*0.6-H28*10+I28*15+J28/200-M28*5</f>
+        <f>C28-D28*20-E28*0.8-F28*0.6-H28*10+I28*15+J28/200-N28*5</f>
         <v/>
       </c>
     </row>
@@ -1842,7 +1842,7 @@
       </c>
       <c r="N29" s="1" t="n"/>
       <c r="O29">
-        <f>C29-D29*20-E29*0.8-F29*0.6-H29*10+I29*15+J29/200-M29*5</f>
+        <f>C29-D29*20-E29*0.8-F29*0.6-H29*10+I29*15+J29/200-N29*5</f>
         <v/>
       </c>
     </row>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="N30" s="1" t="n"/>
       <c r="O30">
-        <f>C30-D30*20-E30*0.8-F30*0.6-H30*10+I30*15+J30/200-M30*5</f>
+        <f>C30-D30*20-E30*0.8-F30*0.6-H30*10+I30*15+J30/200-N30*5</f>
         <v/>
       </c>
     </row>
@@ -1896,7 +1896,7 @@
       <c r="M31" s="1" t="n"/>
       <c r="N31" s="1" t="n"/>
       <c r="O31">
-        <f>C31-D31*20-E31*0.8-F31*0.6-H31*10+I31*15+J31/200-M31*5</f>
+        <f>C31-D31*20-E31*0.8-F31*0.6-H31*10+I31*15+J31/200-N31*5</f>
         <v/>
       </c>
     </row>
@@ -1930,7 +1930,7 @@
       </c>
       <c r="N32" s="1" t="n"/>
       <c r="O32">
-        <f>C32-D32*20-E32*0.8-F32*0.6-H32*10+I32*15+J32/200-M32*5</f>
+        <f>C32-D32*20-E32*0.8-F32*0.6-H32*10+I32*15+J32/200-N32*5</f>
         <v/>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="N33" s="1" t="n"/>
       <c r="O33">
-        <f>C33-D33*20-E33*0.8-F33*0.6-H33*10+I33*15+J33/200-M33*5</f>
+        <f>C33-D33*20-E33*0.8-F33*0.6-H33*10+I33*15+J33/200-N33*5</f>
         <v/>
       </c>
     </row>
@@ -1998,7 +1998,7 @@
       </c>
       <c r="N34" s="1" t="n"/>
       <c r="O34">
-        <f>C34-D34*20-E34*0.8-F34*0.6-H34*10+I34*15+J34/200-M34*5</f>
+        <f>C34-D34*20-E34*0.8-F34*0.6-H34*10+I34*15+J34/200-N34*5</f>
         <v/>
       </c>
     </row>
@@ -2017,12 +2017,28 @@
       <c r="L35" s="1" t="n"/>
       <c r="M35" s="1" t="n"/>
       <c r="N35" s="1" t="n"/>
+      <c r="O35">
+        <f>C35-D35*20-E35*0.8-F35*0.6-H35*10+I35*15+J35/200-N35*5</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n"/>
-      <c r="B36" s="1" t="n"/>
-      <c r="C36" s="1" t="n"/>
-      <c r="D36" s="1" t="n"/>
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>cgr_klra</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="inlineStr">
+        <is>
+          <t>CGR Klra</t>
+        </is>
+      </c>
+      <c r="C36" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D36" s="1" t="n">
+        <v>0.01</v>
+      </c>
       <c r="E36" s="1" t="n"/>
       <c r="F36" s="1" t="n"/>
       <c r="G36" s="1" t="n"/>
@@ -2031,14 +2047,32 @@
       <c r="J36" s="1" t="n"/>
       <c r="K36" s="1" t="n"/>
       <c r="L36" s="1" t="n"/>
-      <c r="M36" s="1" t="n"/>
+      <c r="M36" s="1" t="n">
+        <v>1000</v>
+      </c>
       <c r="N36" s="1" t="n"/>
+      <c r="O36">
+        <f>C36-D36*20-E36*0.8-F36*0.6-H36*10+I36*15+J36/200-N36*5</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n"/>
-      <c r="B37" s="1" t="n"/>
-      <c r="C37" s="1" t="n"/>
-      <c r="D37" s="1" t="n"/>
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>cgr_klra_flipped</t>
+        </is>
+      </c>
+      <c r="B37" s="1" t="inlineStr">
+        <is>
+          <t>CGR Klra Flipped</t>
+        </is>
+      </c>
+      <c r="C37" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D37" s="1" t="n">
+        <v>0.01</v>
+      </c>
       <c r="E37" s="1" t="n"/>
       <c r="F37" s="1" t="n"/>
       <c r="G37" s="1" t="n"/>
@@ -2047,14 +2081,32 @@
       <c r="J37" s="1" t="n"/>
       <c r="K37" s="1" t="n"/>
       <c r="L37" s="1" t="n"/>
-      <c r="M37" s="1" t="n"/>
+      <c r="M37" s="1" t="n">
+        <v>1000</v>
+      </c>
       <c r="N37" s="1" t="n"/>
+      <c r="O37">
+        <f>C37-D37*20-E37*0.8-F37*0.6-H37*10+I37*15+J37/200-N37*5</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n"/>
-      <c r="B38" s="1" t="n"/>
-      <c r="C38" s="1" t="n"/>
-      <c r="D38" s="1" t="n"/>
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>cgr_jolly_roger</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>CGR Jolly Roger</t>
+        </is>
+      </c>
+      <c r="C38" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D38" s="1" t="n">
+        <v>0.01</v>
+      </c>
       <c r="E38" s="1" t="n"/>
       <c r="F38" s="1" t="n"/>
       <c r="G38" s="1" t="n"/>
@@ -2063,14 +2115,32 @@
       <c r="J38" s="1" t="n"/>
       <c r="K38" s="1" t="n"/>
       <c r="L38" s="1" t="n"/>
-      <c r="M38" s="1" t="n"/>
+      <c r="M38" s="1" t="n">
+        <v>1000</v>
+      </c>
       <c r="N38" s="1" t="n"/>
+      <c r="O38">
+        <f>C38-D38*20-E38*0.8-F38*0.6-H38*10+I38*15+J38/200-N38*5</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n"/>
-      <c r="B39" s="1" t="n"/>
-      <c r="C39" s="1" t="n"/>
-      <c r="D39" s="1" t="n"/>
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>cgr_jolly_roger_flipped</t>
+        </is>
+      </c>
+      <c r="B39" s="1" t="inlineStr">
+        <is>
+          <t>CGR Jolly Roger Flipped</t>
+        </is>
+      </c>
+      <c r="C39" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D39" s="1" t="n">
+        <v>0.01</v>
+      </c>
       <c r="E39" s="1" t="n"/>
       <c r="F39" s="1" t="n"/>
       <c r="G39" s="1" t="n"/>
@@ -2079,8 +2149,354 @@
       <c r="J39" s="1" t="n"/>
       <c r="K39" s="1" t="n"/>
       <c r="L39" s="1" t="n"/>
-      <c r="M39" s="1" t="n"/>
+      <c r="M39" s="1" t="n">
+        <v>1000</v>
+      </c>
       <c r="N39" s="1" t="n"/>
+      <c r="O39">
+        <f>C39-D39*20-E39*0.8-F39*0.6-H39*10+I39*15+J39/200-N39*5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr">
+        <is>
+          <t>cgr_ace</t>
+        </is>
+      </c>
+      <c r="B40" s="1" t="inlineStr">
+        <is>
+          <t>CGR Ace Negev</t>
+        </is>
+      </c>
+      <c r="C40" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D40" s="1" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E40" s="1" t="n"/>
+      <c r="F40" s="1" t="n"/>
+      <c r="G40" s="1" t="n"/>
+      <c r="H40" s="1" t="n"/>
+      <c r="I40" s="1" t="n"/>
+      <c r="J40" s="1" t="n"/>
+      <c r="K40" s="1" t="n"/>
+      <c r="L40" s="1" t="n"/>
+      <c r="M40" s="1" t="n">
+        <v>1000</v>
+      </c>
+      <c r="N40" s="1" t="n"/>
+      <c r="O40">
+        <f>C40-D40*20-E40*0.8-F40*0.6-H40*10+I40*15+J40/200-N40*5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>cgr_ace_flipped</t>
+        </is>
+      </c>
+      <c r="B41" s="1" t="inlineStr">
+        <is>
+          <t>CGR Ace Negev Flipped</t>
+        </is>
+      </c>
+      <c r="C41" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D41" s="1" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E41" s="1" t="n"/>
+      <c r="F41" s="1" t="n"/>
+      <c r="G41" s="1" t="n"/>
+      <c r="H41" s="1" t="n"/>
+      <c r="I41" s="1" t="n"/>
+      <c r="J41" s="1" t="n"/>
+      <c r="K41" s="1" t="n"/>
+      <c r="L41" s="1" t="n"/>
+      <c r="M41" s="1" t="n">
+        <v>1000</v>
+      </c>
+      <c r="N41" s="1" t="n"/>
+      <c r="O41">
+        <f>C41-D41*20-E41*0.8-F41*0.6-H41*10+I41*15+J41/200-N41*5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>cgr_abomination</t>
+        </is>
+      </c>
+      <c r="B42" s="1" t="inlineStr">
+        <is>
+          <t>CGR Abomination</t>
+        </is>
+      </c>
+      <c r="C42" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D42" s="1" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E42" s="1" t="n"/>
+      <c r="F42" s="1" t="n"/>
+      <c r="G42" s="1" t="n"/>
+      <c r="H42" s="1" t="n"/>
+      <c r="I42" s="1" t="n"/>
+      <c r="J42" s="1" t="n"/>
+      <c r="K42" s="1" t="n"/>
+      <c r="L42" s="1" t="n"/>
+      <c r="M42" s="1" t="n">
+        <v>1000</v>
+      </c>
+      <c r="N42" s="1" t="n"/>
+      <c r="O42">
+        <f>C42-D42*20-E42*0.8-F42*0.6-H42*10+I42*15+J42/200-N42*5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>cgr_abomination_flipped</t>
+        </is>
+      </c>
+      <c r="B43" s="1" t="inlineStr">
+        <is>
+          <t>CGR Abomination Flipped</t>
+        </is>
+      </c>
+      <c r="C43" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D43" s="1" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E43" s="1" t="n"/>
+      <c r="F43" s="1" t="n"/>
+      <c r="G43" s="1" t="n"/>
+      <c r="H43" s="1" t="n"/>
+      <c r="I43" s="1" t="n"/>
+      <c r="J43" s="1" t="n"/>
+      <c r="K43" s="1" t="n"/>
+      <c r="L43" s="1" t="n"/>
+      <c r="M43" s="1" t="n">
+        <v>1000</v>
+      </c>
+      <c r="N43" s="1" t="n"/>
+      <c r="O43">
+        <f>C43-D43*20-E43*0.8-F43*0.6-H43*10+I43*15+J43/200-N43*5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>cgr_punisher</t>
+        </is>
+      </c>
+      <c r="B44" s="1" t="inlineStr">
+        <is>
+          <t>CGR Punisher</t>
+        </is>
+      </c>
+      <c r="C44" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D44" s="1" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E44" s="1" t="n"/>
+      <c r="F44" s="1" t="n"/>
+      <c r="G44" s="1" t="n"/>
+      <c r="H44" s="1" t="n"/>
+      <c r="I44" s="1" t="n"/>
+      <c r="J44" s="1" t="n"/>
+      <c r="K44" s="1" t="n"/>
+      <c r="L44" s="1" t="n"/>
+      <c r="M44" s="1" t="n">
+        <v>1000</v>
+      </c>
+      <c r="N44" s="1" t="n"/>
+      <c r="O44">
+        <f>C44-D44*20-E44*0.8-F44*0.6-H44*10+I44*15+J44/200-N44*5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>cgr_punisher_flipped</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="inlineStr">
+        <is>
+          <t>CGR Punisher Flipped</t>
+        </is>
+      </c>
+      <c r="C45" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D45" s="1" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E45" s="1" t="n"/>
+      <c r="F45" s="1" t="n"/>
+      <c r="G45" s="1" t="n"/>
+      <c r="H45" s="1" t="n"/>
+      <c r="I45" s="1" t="n"/>
+      <c r="J45" s="1" t="n"/>
+      <c r="K45" s="1" t="n"/>
+      <c r="L45" s="1" t="n"/>
+      <c r="M45" s="1" t="n">
+        <v>1000</v>
+      </c>
+      <c r="N45" s="1" t="n"/>
+      <c r="O45">
+        <f>C45-D45*20-E45*0.8-F45*0.6-H45*10+I45*15+J45/200-N45*5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>cgr_dingler</t>
+        </is>
+      </c>
+      <c r="B46" s="1" t="inlineStr">
+        <is>
+          <t>CGR Dingler</t>
+        </is>
+      </c>
+      <c r="C46" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D46" s="1" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E46" s="1" t="n"/>
+      <c r="F46" s="1" t="n"/>
+      <c r="G46" s="1" t="n"/>
+      <c r="H46" s="1" t="n"/>
+      <c r="I46" s="1" t="n"/>
+      <c r="J46" s="1" t="n"/>
+      <c r="K46" s="1" t="n"/>
+      <c r="L46" s="1" t="n"/>
+      <c r="M46" s="1" t="n">
+        <v>1000</v>
+      </c>
+      <c r="N46" s="1" t="n"/>
+      <c r="O46">
+        <f>C46-D46*20-E46*0.8-F46*0.6-H46*10+I46*15+J46/200-N46*5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>cgr_dingler_flipped</t>
+        </is>
+      </c>
+      <c r="B47" s="1" t="inlineStr">
+        <is>
+          <t>CGR Dingler Flipped</t>
+        </is>
+      </c>
+      <c r="C47" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D47" s="1" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E47" s="1" t="n"/>
+      <c r="F47" s="1" t="n"/>
+      <c r="G47" s="1" t="n"/>
+      <c r="H47" s="1" t="n"/>
+      <c r="I47" s="1" t="n"/>
+      <c r="J47" s="1" t="n"/>
+      <c r="K47" s="1" t="n"/>
+      <c r="L47" s="1" t="n"/>
+      <c r="M47" s="1" t="n">
+        <v>1000</v>
+      </c>
+      <c r="N47" s="1" t="n"/>
+      <c r="O47">
+        <f>C47-D47*20-E47*0.8-F47*0.6-H47*10+I47*15+J47/200-N47*5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>cgr_aeon</t>
+        </is>
+      </c>
+      <c r="B48" s="1" t="inlineStr">
+        <is>
+          <t>CGR Aeon</t>
+        </is>
+      </c>
+      <c r="C48" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D48" s="1" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E48" s="1" t="n"/>
+      <c r="F48" s="1" t="n"/>
+      <c r="G48" s="1" t="n"/>
+      <c r="H48" s="1" t="n"/>
+      <c r="I48" s="1" t="n"/>
+      <c r="J48" s="1" t="n"/>
+      <c r="K48" s="1" t="n"/>
+      <c r="L48" s="1" t="n"/>
+      <c r="M48" s="1" t="n">
+        <v>1000</v>
+      </c>
+      <c r="N48" s="1" t="n"/>
+      <c r="O48">
+        <f>C48-D48*20-E48*0.8-F48*0.6-H48*10+I48*15+J48/200-N48*5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>cgr_aeon_flipped</t>
+        </is>
+      </c>
+      <c r="B49" s="1" t="inlineStr">
+        <is>
+          <t>CGR Aeon Flipped</t>
+        </is>
+      </c>
+      <c r="C49" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D49" s="1" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E49" s="1" t="n"/>
+      <c r="F49" s="1" t="n"/>
+      <c r="G49" s="1" t="n"/>
+      <c r="H49" s="1" t="n"/>
+      <c r="I49" s="1" t="n"/>
+      <c r="J49" s="1" t="n"/>
+      <c r="K49" s="1" t="n"/>
+      <c r="L49" s="1" t="n"/>
+      <c r="M49" s="1" t="n">
+        <v>1000</v>
+      </c>
+      <c r="N49" s="1" t="n"/>
+      <c r="O49">
+        <f>C49-D49*20-E49*0.8-F49*0.6-H49*10+I49*15+J49/200-N49*5</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
rail panels: 1 ergo per 0.04 weight, cgr/arrow ax/veles weights, per-slot pricing for magtap type1 and ecmr
</commit_message>
<xml_diff>
--- a/changes/rail-panels.xlsx
+++ b/changes/rail-panels.xlsx
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>0.66</v>
+        <v>0.5</v>
       </c>
       <c r="D3" s="1" t="n">
         <v>0.02</v>
@@ -1058,7 +1058,7 @@
         </is>
       </c>
       <c r="C4" s="1" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>0.03</v>
@@ -1092,7 +1092,7 @@
         </is>
       </c>
       <c r="C5" s="1" t="n">
-        <v>1.33</v>
+        <v>1</v>
       </c>
       <c r="D5" s="1" t="n">
         <v>0.04</v>
@@ -1126,7 +1126,7 @@
         </is>
       </c>
       <c r="C6" s="1" t="n">
-        <v>1.66</v>
+        <v>1.25</v>
       </c>
       <c r="D6" s="1" t="n">
         <v>0.05</v>
@@ -1160,7 +1160,7 @@
         </is>
       </c>
       <c r="C7" s="1" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D7" s="1" t="n">
         <v>0.06</v>
@@ -1194,7 +1194,7 @@
         </is>
       </c>
       <c r="C8" s="1" t="n">
-        <v>2.33</v>
+        <v>1.75</v>
       </c>
       <c r="D8" s="1" t="n">
         <v>0.07000000000000001</v>
@@ -1248,7 +1248,7 @@
         </is>
       </c>
       <c r="C10" s="1" t="n">
-        <v>0.33</v>
+        <v>0.25</v>
       </c>
       <c r="D10" s="1" t="n">
         <v>0.01</v>
@@ -1282,7 +1282,7 @@
         </is>
       </c>
       <c r="C11" s="1" t="n">
-        <v>0.66</v>
+        <v>0.5</v>
       </c>
       <c r="D11" s="1" t="n">
         <v>0.02</v>
@@ -1316,7 +1316,7 @@
         </is>
       </c>
       <c r="C12" s="1" t="n">
-        <v>1.33</v>
+        <v>1</v>
       </c>
       <c r="D12" s="1" t="n">
         <v>0.04</v>
@@ -1350,7 +1350,7 @@
         </is>
       </c>
       <c r="C13" s="1" t="n">
-        <v>2.33</v>
+        <v>1.75</v>
       </c>
       <c r="D13" s="1" t="n">
         <v>0.07000000000000001</v>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="C15" s="1" t="n">
-        <v>1.33</v>
+        <v>1</v>
       </c>
       <c r="D15" s="1" t="n">
         <v>0.04</v>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="C16" s="1" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D16" s="1" t="n">
         <v>0.06</v>
@@ -1472,7 +1472,7 @@
         </is>
       </c>
       <c r="C17" s="1" t="n">
-        <v>2.66</v>
+        <v>2</v>
       </c>
       <c r="D17" s="1" t="n">
         <v>0.08</v>
@@ -1526,7 +1526,7 @@
         </is>
       </c>
       <c r="C19" s="1" t="n">
-        <v>0.66</v>
+        <v>0.5</v>
       </c>
       <c r="D19" s="1" t="n">
         <v>0.02</v>
@@ -1563,7 +1563,7 @@
         <v>1</v>
       </c>
       <c r="D20" s="1" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="E20" s="1" t="n"/>
       <c r="F20" s="1" t="n"/>
@@ -1614,10 +1614,10 @@
         </is>
       </c>
       <c r="C22" s="1" t="n">
-        <v>0.66</v>
+        <v>0.75</v>
       </c>
       <c r="D22" s="1" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="E22" s="1" t="n"/>
       <c r="F22" s="1" t="n"/>
@@ -1628,7 +1628,7 @@
       <c r="K22" s="1" t="n"/>
       <c r="L22" s="1" t="n"/>
       <c r="M22" s="1" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="N22" s="1" t="n"/>
       <c r="O22">
@@ -1648,10 +1648,10 @@
         </is>
       </c>
       <c r="C23" s="1" t="n">
-        <v>0.66</v>
+        <v>0.75</v>
       </c>
       <c r="D23" s="1" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="E23" s="1" t="n"/>
       <c r="F23" s="1" t="n"/>
@@ -1662,7 +1662,7 @@
       <c r="K23" s="1" t="n"/>
       <c r="L23" s="1" t="n"/>
       <c r="M23" s="1" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="N23" s="1" t="n"/>
       <c r="O23">
@@ -1702,7 +1702,7 @@
         </is>
       </c>
       <c r="C25" s="1" t="n">
-        <v>0.66</v>
+        <v>0.5</v>
       </c>
       <c r="D25" s="1" t="n">
         <v>0.02</v>
@@ -1736,7 +1736,7 @@
         </is>
       </c>
       <c r="C26" s="1" t="n">
-        <v>1.66</v>
+        <v>1.25</v>
       </c>
       <c r="D26" s="1" t="n">
         <v>0.05</v>
@@ -1770,7 +1770,7 @@
         </is>
       </c>
       <c r="C27" s="1" t="n">
-        <v>3</v>
+        <v>2.25</v>
       </c>
       <c r="D27" s="1" t="n">
         <v>0.09</v>
@@ -1784,7 +1784,7 @@
       <c r="K27" s="1" t="n"/>
       <c r="L27" s="1" t="n"/>
       <c r="M27" s="1" t="n">
-        <v>900</v>
+        <v>600</v>
       </c>
       <c r="N27" s="1" t="n"/>
       <c r="O27">
@@ -1824,7 +1824,7 @@
         </is>
       </c>
       <c r="C29" s="1" t="n">
-        <v>0.33</v>
+        <v>0.25</v>
       </c>
       <c r="D29" s="1" t="n">
         <v>0.01</v>
@@ -1858,7 +1858,7 @@
         </is>
       </c>
       <c r="C30" s="1" t="n">
-        <v>0.66</v>
+        <v>0.5</v>
       </c>
       <c r="D30" s="1" t="n">
         <v>0.02</v>
@@ -1912,7 +1912,7 @@
         </is>
       </c>
       <c r="C32" s="1" t="n">
-        <v>0.33</v>
+        <v>0.25</v>
       </c>
       <c r="D32" s="1" t="n">
         <v>0.01</v>
@@ -1946,7 +1946,7 @@
         </is>
       </c>
       <c r="C33" s="1" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="D33" s="1" t="n">
         <v>0.03</v>
@@ -1960,7 +1960,7 @@
       <c r="K33" s="1" t="n"/>
       <c r="L33" s="1" t="n"/>
       <c r="M33" s="1" t="n">
-        <v>600</v>
+        <v>400</v>
       </c>
       <c r="N33" s="1" t="n"/>
       <c r="O33">
@@ -1980,7 +1980,7 @@
         </is>
       </c>
       <c r="C34" s="1" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D34" s="1" t="n">
         <v>0.06</v>
@@ -1994,7 +1994,7 @@
       <c r="K34" s="1" t="n"/>
       <c r="L34" s="1" t="n"/>
       <c r="M34" s="1" t="n">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="N34" s="1" t="n"/>
       <c r="O34">
@@ -2034,10 +2034,10 @@
         </is>
       </c>
       <c r="C36" s="1" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="D36" s="1" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="E36" s="1" t="n"/>
       <c r="F36" s="1" t="n"/>
@@ -2068,10 +2068,10 @@
         </is>
       </c>
       <c r="C37" s="1" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="D37" s="1" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="E37" s="1" t="n"/>
       <c r="F37" s="1" t="n"/>
@@ -2102,10 +2102,10 @@
         </is>
       </c>
       <c r="C38" s="1" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="D38" s="1" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="E38" s="1" t="n"/>
       <c r="F38" s="1" t="n"/>
@@ -2136,10 +2136,10 @@
         </is>
       </c>
       <c r="C39" s="1" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="D39" s="1" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="E39" s="1" t="n"/>
       <c r="F39" s="1" t="n"/>
@@ -2170,10 +2170,10 @@
         </is>
       </c>
       <c r="C40" s="1" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="D40" s="1" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="E40" s="1" t="n"/>
       <c r="F40" s="1" t="n"/>
@@ -2204,10 +2204,10 @@
         </is>
       </c>
       <c r="C41" s="1" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="D41" s="1" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="E41" s="1" t="n"/>
       <c r="F41" s="1" t="n"/>
@@ -2238,10 +2238,10 @@
         </is>
       </c>
       <c r="C42" s="1" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="D42" s="1" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="E42" s="1" t="n"/>
       <c r="F42" s="1" t="n"/>
@@ -2272,10 +2272,10 @@
         </is>
       </c>
       <c r="C43" s="1" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="D43" s="1" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="E43" s="1" t="n"/>
       <c r="F43" s="1" t="n"/>
@@ -2306,10 +2306,10 @@
         </is>
       </c>
       <c r="C44" s="1" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="D44" s="1" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="E44" s="1" t="n"/>
       <c r="F44" s="1" t="n"/>
@@ -2340,10 +2340,10 @@
         </is>
       </c>
       <c r="C45" s="1" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="D45" s="1" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="E45" s="1" t="n"/>
       <c r="F45" s="1" t="n"/>
@@ -2374,10 +2374,10 @@
         </is>
       </c>
       <c r="C46" s="1" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="D46" s="1" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="E46" s="1" t="n"/>
       <c r="F46" s="1" t="n"/>
@@ -2408,10 +2408,10 @@
         </is>
       </c>
       <c r="C47" s="1" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="D47" s="1" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="E47" s="1" t="n"/>
       <c r="F47" s="1" t="n"/>
@@ -2442,10 +2442,10 @@
         </is>
       </c>
       <c r="C48" s="1" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="D48" s="1" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="E48" s="1" t="n"/>
       <c r="F48" s="1" t="n"/>
@@ -2476,10 +2476,10 @@
         </is>
       </c>
       <c r="C49" s="1" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="D49" s="1" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="E49" s="1" t="n"/>
       <c r="F49" s="1" t="n"/>

</xml_diff>